<commit_message>
Commit arquivos MBA Eng Dados
</commit_message>
<xml_diff>
--- a/Lista Presença Alunos.xlsx
+++ b/Lista Presença Alunos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Temp\Python_YT\Git\sirius_mba_engenharia_dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFFE944F-888E-4FE4-A25F-E14413762046}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59B4269A-6C88-4E6D-B71D-6481D800BC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="18">
   <si>
     <t>Aluno</t>
   </si>
@@ -75,6 +75,12 @@
   </si>
   <si>
     <t>Alunos Pós - Listagem de Presença</t>
+  </si>
+  <si>
+    <t>Modelagem Dados</t>
+  </si>
+  <si>
+    <t>SQL</t>
   </si>
 </sst>
 </file>
@@ -152,22 +158,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -178,6 +177,16 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -397,371 +406,371 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q46"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="17" width="10.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A1" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+    </row>
+    <row r="2" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+    </row>
+    <row r="3" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="8">
+      <c r="C3" s="5">
         <v>45540</v>
       </c>
-      <c r="D3" s="8">
+      <c r="D3" s="5">
         <v>45545</v>
       </c>
-      <c r="E3" s="8">
+      <c r="E3" s="5">
         <v>45547</v>
       </c>
-      <c r="F3" s="8">
+      <c r="F3" s="5">
         <v>45553</v>
       </c>
-      <c r="G3" s="8">
+      <c r="G3" s="5">
         <v>45559</v>
       </c>
-      <c r="H3" s="8">
+      <c r="H3" s="5">
         <v>45561</v>
       </c>
-      <c r="I3" s="8">
+      <c r="I3" s="5">
         <v>45566</v>
       </c>
-      <c r="J3" s="9">
+      <c r="J3" s="6">
         <v>45568</v>
       </c>
-      <c r="K3" s="9">
+      <c r="K3" s="6">
         <v>45573</v>
       </c>
-      <c r="L3" s="10">
+      <c r="L3" s="7">
         <v>45575</v>
       </c>
-      <c r="M3" s="10">
+      <c r="M3" s="7">
         <v>45581</v>
       </c>
-      <c r="N3" s="10">
+      <c r="N3" s="7">
         <v>45587</v>
       </c>
-      <c r="O3" s="10">
+      <c r="O3" s="7">
         <v>45588</v>
       </c>
-      <c r="P3" s="10">
+      <c r="P3" s="7">
         <v>45589</v>
       </c>
-      <c r="Q3" s="10">
+      <c r="Q3" s="7">
         <v>45594</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="11"/>
-      <c r="F4" s="11"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+      <c r="C4" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
+      <c r="I4" s="8"/>
+      <c r="J4" s="8"/>
+      <c r="K4" s="8"/>
+      <c r="L4" s="8"/>
+      <c r="M4" s="8"/>
+      <c r="N4" s="8"/>
+      <c r="O4" s="8"/>
+      <c r="P4" s="8"/>
+      <c r="Q4" s="8"/>
+    </row>
+    <row r="5" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="11"/>
-      <c r="F5" s="11"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="11"/>
-      <c r="I5" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A6" s="7" t="s">
+      <c r="C5" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
+      <c r="I5" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="J5" s="8"/>
+      <c r="K5" s="8"/>
+      <c r="L5" s="8"/>
+      <c r="M5" s="8"/>
+      <c r="N5" s="8"/>
+      <c r="O5" s="8"/>
+      <c r="P5" s="8"/>
+      <c r="Q5" s="8"/>
+    </row>
+    <row r="6" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="E6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="H6" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A7" s="7" t="s">
+      <c r="C6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
+    </row>
+    <row r="7" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" s="11"/>
-      <c r="G7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I7" s="11"/>
-      <c r="J7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A8" s="7" t="s">
+      <c r="C7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I7" s="8"/>
+      <c r="J7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="M7" s="8"/>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="J8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="M8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="N8" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
+      <c r="C8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D8" s="8"/>
+      <c r="E8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="N8" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
+    </row>
+    <row r="9" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="11"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I9" s="11"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="B10" s="7" t="s">
+      <c r="C9" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
+      <c r="H9" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I9" s="8"/>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="F10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="G10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="H10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="I10" s="11"/>
-      <c r="J10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="M10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="N10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="O10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="P10" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="11" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A11" s="7" t="s">
+      <c r="C10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="G10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="I10" s="8"/>
+      <c r="J10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="N10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="P10" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="Q10" s="8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="E11" s="11"/>
-      <c r="F11" s="11"/>
-      <c r="G11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="H11" s="11"/>
-      <c r="I11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="J11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="K11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="L11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="M11" s="11" t="s">
-        <v>4</v>
-      </c>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
+      <c r="C11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="H11" s="8"/>
+      <c r="I11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
     </row>
     <row r="14" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
     </row>
     <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -860,6 +869,204 @@
       </c>
       <c r="C24" s="1">
         <v>8</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C29" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C30" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C31" s="1">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C32" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C33" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C34" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C39" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C40" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C41" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C42" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C43" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C44" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C45" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C46" s="1">
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>